<commit_message>
fix(checkout): đồng bộ text lỗi SĐT "Số điện thoại không đúng" (BA 2026-06-11)
- Cập nhật message lỗi định dạng SĐT từ "không hợp lệ"/"chưa đúng" → "không đúng"
  trong automation specs (ckcommon.shared, ultrafast) và script gen (gen_tc_checkout,
  gen_tc_ultrafast) + regen Excel TC checkout/dangkyUF
- Cập nhật tài liệu analyze-requirement checkout (MEMORY, traceability, risk, scenario map)
- sync_tc_checkout.py: bổ sung xử lý sync kết quả
- settings.local.json: thêm allowed bash/read permissions

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ecom-pdh/03_test-cases/functional/chucnang_checkout/AI_ISC_ecom-pdh_v1.1_TC_checkout_v1.2.xlsx
+++ b/ecom-pdh/03_test-cases/functional/chucnang_checkout/AI_ISC_ecom-pdh_v1.1_TC_checkout_v1.2.xlsx
@@ -812,12 +812,12 @@
       <c r="J7" s="36" t="n"/>
       <c r="K7" s="36" t="n"/>
       <c r="L7" s="37" t="n"/>
-      <c r="M7" s="38" t="inlineStr">
+      <c r="M7" s="39" t="inlineStr">
         <is>
           <t>Camera</t>
         </is>
       </c>
-      <c r="Q7" s="38" t="inlineStr">
+      <c r="Q7" s="39" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
@@ -857,42 +857,42 @@
           <t>Ghi Chú</t>
         </is>
       </c>
-      <c r="M8" s="38" t="inlineStr">
+      <c r="M8" s="39" t="inlineStr">
         <is>
           <t>Kết Quả Thực Hiện</t>
         </is>
       </c>
-      <c r="N8" s="38" t="inlineStr">
+      <c r="N8" s="39" t="inlineStr">
         <is>
           <t>Người Thực Hiện</t>
         </is>
       </c>
-      <c r="O8" s="38" t="inlineStr">
+      <c r="O8" s="39" t="inlineStr">
         <is>
           <t>ID Bugs</t>
         </is>
       </c>
-      <c r="P8" s="38" t="inlineStr">
+      <c r="P8" s="39" t="inlineStr">
         <is>
           <t>Ghi Chú</t>
         </is>
       </c>
-      <c r="Q8" s="38" t="inlineStr">
+      <c r="Q8" s="39" t="inlineStr">
         <is>
           <t>Kết Quả Thực Hiện</t>
         </is>
       </c>
-      <c r="R8" s="38" t="inlineStr">
+      <c r="R8" s="39" t="inlineStr">
         <is>
           <t>Người Thực Hiện</t>
         </is>
       </c>
-      <c r="S8" s="38" t="inlineStr">
+      <c r="S8" s="39" t="inlineStr">
         <is>
           <t>ID Bugs</t>
         </is>
       </c>
-      <c r="T8" s="38" t="inlineStr">
+      <c r="T8" s="39" t="inlineStr">
         <is>
           <t>Ghi Chú</t>
         </is>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="G23" s="44" t="inlineStr">
         <is>
-          <t>Hiển thị "Số điện thoại không hợp lệ."</t>
+          <t>Hiển thị "Số điện thoại không đúng."</t>
         </is>
       </c>
       <c r="H23" s="43" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="G24" s="44" t="inlineStr">
         <is>
-          <t>Hiển thị "Số điện thoại không hợp lệ."</t>
+          <t>Hiển thị "Số điện thoại không đúng."</t>
         </is>
       </c>
       <c r="H24" s="43" t="inlineStr">
@@ -6742,7 +6742,6 @@
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="B30:L30"/>
-    <mergeCell ref="B14:L14"/>
     <mergeCell ref="B9:L9"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="B20:L20"/>
@@ -6752,12 +6751,13 @@
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="G7:G8"/>
     <mergeCell ref="F7:F8"/>
+    <mergeCell ref="B14:L14"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="I7:L7"/>
     <mergeCell ref="B10:L10"/>
-    <mergeCell ref="B17:L17"/>
     <mergeCell ref="B23:L23"/>
     <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B17:L17"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>